<commit_message>
Normalize docente excel data and extend import flow
</commit_message>
<xml_diff>
--- a/Lista Administradores FICCT_poblado.xlsx
+++ b/Lista Administradores FICCT_poblado.xlsx
@@ -1,34 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29930"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_630234F90D81DB95DA2FC29280913E03AFCAB5F7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C216BFA-68C1-4B94-8769-0C34F85A9027}"/>
-  <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
-  <sheets>
-    <sheet name="Docente" sheetId="1" r:id="rId1"/>
-    <sheet name="Estudiante" sheetId="2" r:id="rId2"/>
-  </sheets>
-  <calcPr calcId="191028" refMode="R1C1" iterateCount="0" calcOnSave="0" concurrentCalc="0"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
-</workbook>
+<ns0:workbook xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:ns5="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:ns6="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ns7="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:ns8="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" ns1:Ignorable="x15 xr xr6 xr10 xr2">
+  <ns0:fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29930"/>
+  <ns0:workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
+  <ns2:revisionPtr revIDLastSave="1" documentId="11_630234F90D81DB95DA2FC29280913E03AFCAB5F7" ns3:coauthVersionLast="47" ns3:coauthVersionMax="47" ns4:uidLastSave="{0C216BFA-68C1-4B94-8769-0C34F85A9027}"/>
+  <ns0:bookViews>
+    <ns0:workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" ns5:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </ns0:bookViews>
+  <ns0:sheets>
+    <ns0:sheet name="Docente" sheetId="1" ns6:id="rId1"/>
+  </ns0:sheets>
+  <ns0:calcPr calcId="191028" refMode="R1C1" iterateCount="0" calcOnSave="0" concurrentCalc="0"/>
+  <ns0:extLst>
+    <ns0:ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <ns7:workbookPr chartTrackingRefBase="1"/>
+    </ns0:ext>
+    <ns0:ext uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <ns8:calcFeatures>
+        <ns8:feature name="microsoft.com:RD"/>
+        <ns8:feature name="microsoft.com:Single"/>
+        <ns8:feature name="microsoft.com:FV"/>
+        <ns8:feature name="microsoft.com:CNMTM"/>
+        <ns8:feature name="microsoft.com:LET_WF"/>
+        <ns8:feature name="microsoft.com:LAMBDA_WF"/>
+        <ns8:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </ns8:calcFeatures>
+    </ns0:ext>
+  </ns0:extLst>
+</ns0:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2862,7 +2861,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L225"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -2943,8 +2942,10 @@
       <c r="C3" t="s">
         <v>14</v>
       </c>
-      <c r="D3" t="s">
-        <v>20</v>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>300000000</t>
+        </is>
       </c>
       <c r="E3" t="s">
         <v>16</v>
@@ -2958,8 +2959,10 @@
       <c r="J3" t="s">
         <v>21</v>
       </c>
-      <c r="L3" t="s">
-        <v>22</v>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>flores.oscar@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -3085,8 +3088,10 @@
       <c r="C8" t="s">
         <v>29</v>
       </c>
-      <c r="D8" t="s">
-        <v>44</v>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>300000003</t>
+        </is>
       </c>
       <c r="E8" t="s">
         <v>31</v>
@@ -3100,8 +3105,10 @@
       <c r="J8" t="s">
         <v>45</v>
       </c>
-      <c r="L8" t="s">
-        <v>46</v>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>cortez.martin@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -3114,8 +3121,10 @@
       <c r="C9" t="s">
         <v>29</v>
       </c>
-      <c r="D9" t="s">
-        <v>47</v>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>300000003</t>
+        </is>
       </c>
       <c r="E9" t="s">
         <v>31</v>
@@ -3129,8 +3138,10 @@
       <c r="J9" t="s">
         <v>37</v>
       </c>
-      <c r="L9" t="s">
-        <v>48</v>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>cortez.martin@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -3143,8 +3154,10 @@
       <c r="C10" t="s">
         <v>29</v>
       </c>
-      <c r="D10" t="s">
-        <v>49</v>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>300000003</t>
+        </is>
       </c>
       <c r="E10" t="s">
         <v>31</v>
@@ -3158,8 +3171,10 @@
       <c r="J10" t="s">
         <v>21</v>
       </c>
-      <c r="L10" t="s">
-        <v>50</v>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>cortez.martin@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -3198,8 +3213,10 @@
       <c r="C12" t="s">
         <v>52</v>
       </c>
-      <c r="D12" t="s">
-        <v>56</v>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>300000009</t>
+        </is>
       </c>
       <c r="E12" t="s">
         <v>54</v>
@@ -3213,8 +3230,10 @@
       <c r="J12" t="s">
         <v>21</v>
       </c>
-      <c r="L12" t="s">
-        <v>57</v>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>monrroy.fernando@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -3227,8 +3246,10 @@
       <c r="C13" t="s">
         <v>60</v>
       </c>
-      <c r="D13" t="s">
-        <v>61</v>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>300000009</t>
+        </is>
       </c>
       <c r="E13" t="s">
         <v>54</v>
@@ -3242,8 +3263,10 @@
       <c r="J13" t="s">
         <v>45</v>
       </c>
-      <c r="L13" t="s">
-        <v>62</v>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>monrroy.fernando@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -3311,8 +3334,10 @@
       <c r="C16" t="s">
         <v>70</v>
       </c>
-      <c r="D16" t="s">
-        <v>74</v>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>300000013</t>
+        </is>
       </c>
       <c r="E16" t="s">
         <v>72</v>
@@ -3323,8 +3348,10 @@
       <c r="I16" t="s">
         <v>75</v>
       </c>
-      <c r="L16" t="s">
-        <v>76</v>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>hinojosa.said@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -3337,8 +3364,10 @@
       <c r="C17" t="s">
         <v>70</v>
       </c>
-      <c r="D17" t="s">
-        <v>79</v>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>300000013</t>
+        </is>
       </c>
       <c r="E17" t="s">
         <v>72</v>
@@ -3352,8 +3381,10 @@
       <c r="J17" t="s">
         <v>80</v>
       </c>
-      <c r="L17" t="s">
-        <v>81</v>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>hinojosa.said@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -3366,8 +3397,10 @@
       <c r="C18" t="s">
         <v>70</v>
       </c>
-      <c r="D18" t="s">
-        <v>82</v>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>300000013</t>
+        </is>
       </c>
       <c r="E18" t="s">
         <v>72</v>
@@ -3381,8 +3414,10 @@
       <c r="J18" t="s">
         <v>80</v>
       </c>
-      <c r="L18" t="s">
-        <v>83</v>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>hinojosa.said@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="19" spans="1:12">
@@ -3395,14 +3430,18 @@
       <c r="C19" t="s">
         <v>70</v>
       </c>
-      <c r="D19" t="s">
-        <v>85</v>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>300000013</t>
+        </is>
       </c>
       <c r="E19" t="s">
         <v>72</v>
       </c>
-      <c r="L19" t="s">
-        <v>86</v>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>hinojosa.said@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="20" spans="1:12">
@@ -3473,8 +3512,10 @@
       <c r="C22" t="s">
         <v>99</v>
       </c>
-      <c r="D22" t="s">
-        <v>100</v>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>300000018</t>
+        </is>
       </c>
       <c r="E22" t="s">
         <v>90</v>
@@ -3488,8 +3529,10 @@
       <c r="J22" t="s">
         <v>45</v>
       </c>
-      <c r="L22" t="s">
-        <v>101</v>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>veizaga.obed@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="23" spans="1:12">
@@ -3502,8 +3545,10 @@
       <c r="C23" t="s">
         <v>99</v>
       </c>
-      <c r="D23" t="s">
-        <v>102</v>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>300000018</t>
+        </is>
       </c>
       <c r="E23" t="s">
         <v>90</v>
@@ -3514,8 +3559,10 @@
       <c r="I23" t="s">
         <v>42</v>
       </c>
-      <c r="L23" t="s">
-        <v>103</v>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>veizaga.obed@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="24" spans="1:12">
@@ -3574,8 +3621,10 @@
       <c r="C26" t="s">
         <v>109</v>
       </c>
-      <c r="D26" t="s">
-        <v>114</v>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>300000023</t>
+        </is>
       </c>
       <c r="E26" t="s">
         <v>111</v>
@@ -3586,8 +3635,10 @@
       <c r="I26" t="s">
         <v>75</v>
       </c>
-      <c r="L26" t="s">
-        <v>115</v>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>perez.ubaldo@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="27" spans="1:12">
@@ -3973,8 +4024,10 @@
       <c r="C41" t="s">
         <v>180</v>
       </c>
-      <c r="D41" t="s">
-        <v>181</v>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>300000029</t>
+        </is>
       </c>
       <c r="E41" t="s">
         <v>138</v>
@@ -3985,8 +4038,10 @@
       <c r="J41" t="s">
         <v>135</v>
       </c>
-      <c r="L41" t="s">
-        <v>182</v>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>morales.magaly@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="42" spans="1:12">
@@ -4054,8 +4109,10 @@
       <c r="C44" t="s">
         <v>180</v>
       </c>
-      <c r="D44" t="s">
-        <v>192</v>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>300000036</t>
+        </is>
       </c>
       <c r="E44" t="s">
         <v>168</v>
@@ -4066,8 +4123,10 @@
       <c r="I44" t="s">
         <v>75</v>
       </c>
-      <c r="L44" t="s">
-        <v>193</v>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>calizaya.fidel@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="45" spans="1:12">
@@ -4109,8 +4168,10 @@
       <c r="C46" t="s">
         <v>198</v>
       </c>
-      <c r="D46" t="s">
-        <v>199</v>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>300000026</t>
+        </is>
       </c>
       <c r="E46" t="s">
         <v>125</v>
@@ -4124,8 +4185,10 @@
       <c r="K46" t="s">
         <v>21</v>
       </c>
-      <c r="L46" t="s">
-        <v>200</v>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>carreno.andres@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="47" spans="1:12">
@@ -4222,8 +4285,10 @@
       <c r="C50" t="s">
         <v>210</v>
       </c>
-      <c r="D50" t="s">
-        <v>214</v>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>300000000</t>
+        </is>
       </c>
       <c r="E50" t="s">
         <v>16</v>
@@ -4237,8 +4302,10 @@
       <c r="J50" t="s">
         <v>45</v>
       </c>
-      <c r="L50" t="s">
-        <v>215</v>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>flores.oscar@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="51" spans="1:12">
@@ -4352,8 +4419,10 @@
       <c r="C55" t="s">
         <v>240</v>
       </c>
-      <c r="D55" t="s">
-        <v>241</v>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>300000013</t>
+        </is>
       </c>
       <c r="E55" t="s">
         <v>72</v>
@@ -4364,8 +4433,10 @@
       <c r="I55" t="s">
         <v>21</v>
       </c>
-      <c r="L55" t="s">
-        <v>242</v>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>hinojosa.said@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="56" spans="1:12">
@@ -4407,8 +4478,10 @@
       <c r="C57" t="s">
         <v>244</v>
       </c>
-      <c r="D57" t="s">
-        <v>248</v>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>300000054</t>
+        </is>
       </c>
       <c r="E57" t="s">
         <v>246</v>
@@ -4422,8 +4495,10 @@
       <c r="J57" t="s">
         <v>32</v>
       </c>
-      <c r="L57" t="s">
-        <v>249</v>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>terrazas.ricardo@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="58" spans="1:12">
@@ -4436,8 +4511,10 @@
       <c r="C58" t="s">
         <v>252</v>
       </c>
-      <c r="D58" t="s">
-        <v>253</v>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>300000033</t>
+        </is>
       </c>
       <c r="E58" t="s">
         <v>155</v>
@@ -4448,8 +4525,10 @@
       <c r="I58" t="s">
         <v>147</v>
       </c>
-      <c r="L58" t="s">
-        <v>254</v>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>miranda.carlos@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="59" spans="1:12">
@@ -4488,8 +4567,10 @@
       <c r="C60" t="s">
         <v>252</v>
       </c>
-      <c r="D60" t="s">
-        <v>259</v>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>300000057</t>
+        </is>
       </c>
       <c r="E60" t="s">
         <v>257</v>
@@ -4500,8 +4581,10 @@
       <c r="I60" t="s">
         <v>260</v>
       </c>
-      <c r="L60" t="s">
-        <v>261</v>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>grageda.wilson@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="61" spans="1:12">
@@ -4514,8 +4597,10 @@
       <c r="C61" t="s">
         <v>252</v>
       </c>
-      <c r="D61" t="s">
-        <v>262</v>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>300000035</t>
+        </is>
       </c>
       <c r="E61" t="s">
         <v>164</v>
@@ -4526,8 +4611,10 @@
       <c r="I61" t="s">
         <v>260</v>
       </c>
-      <c r="L61" t="s">
-        <v>263</v>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>avendano.eudal@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="62" spans="1:12">
@@ -4566,8 +4653,10 @@
       <c r="C63" t="s">
         <v>270</v>
       </c>
-      <c r="D63" t="s">
-        <v>271</v>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>300000031</t>
+        </is>
       </c>
       <c r="E63" t="s">
         <v>146</v>
@@ -4578,8 +4667,10 @@
       <c r="J63" t="s">
         <v>273</v>
       </c>
-      <c r="L63" t="s">
-        <v>274</v>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>siles.felix@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="64" spans="1:12">
@@ -4670,8 +4761,10 @@
       <c r="C67" t="s">
         <v>281</v>
       </c>
-      <c r="D67" t="s">
-        <v>288</v>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>300000063</t>
+        </is>
       </c>
       <c r="E67" t="s">
         <v>283</v>
@@ -4682,8 +4775,10 @@
       <c r="I67" t="s">
         <v>272</v>
       </c>
-      <c r="L67" t="s">
-        <v>289</v>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>lopez.milton@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="68" spans="1:12">
@@ -4722,8 +4817,10 @@
       <c r="C69" t="s">
         <v>295</v>
       </c>
-      <c r="D69" t="s">
-        <v>296</v>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>300000066</t>
+        </is>
       </c>
       <c r="E69" t="s">
         <v>291</v>
@@ -4734,8 +4831,10 @@
       <c r="I69" t="s">
         <v>42</v>
       </c>
-      <c r="L69" t="s">
-        <v>297</v>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>peinado.carlos@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="70" spans="1:12">
@@ -4829,8 +4928,10 @@
       <c r="C73" t="s">
         <v>306</v>
       </c>
-      <c r="D73" t="s">
-        <v>310</v>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>300000004</t>
+        </is>
       </c>
       <c r="E73" t="s">
         <v>36</v>
@@ -4844,8 +4945,10 @@
       <c r="J73" t="s">
         <v>45</v>
       </c>
-      <c r="L73" t="s">
-        <v>311</v>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>gutierrez.esther@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="74" spans="1:12">
@@ -4858,8 +4961,10 @@
       <c r="C74" t="s">
         <v>306</v>
       </c>
-      <c r="D74" t="s">
-        <v>312</v>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>300000004</t>
+        </is>
       </c>
       <c r="E74" t="s">
         <v>36</v>
@@ -4873,8 +4978,10 @@
       <c r="J74" t="s">
         <v>96</v>
       </c>
-      <c r="L74" t="s">
-        <v>313</v>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>gutierrez.esther@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="75" spans="1:12">
@@ -4887,8 +4994,10 @@
       <c r="C75" t="s">
         <v>306</v>
       </c>
-      <c r="D75" t="s">
-        <v>314</v>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>300000070</t>
+        </is>
       </c>
       <c r="E75" t="s">
         <v>308</v>
@@ -4902,8 +5011,10 @@
       <c r="J75" t="s">
         <v>45</v>
       </c>
-      <c r="L75" t="s">
-        <v>315</v>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>martinez.mirna@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="76" spans="1:12">
@@ -4942,8 +5053,10 @@
       <c r="C77" t="s">
         <v>306</v>
       </c>
-      <c r="D77" t="s">
-        <v>319</v>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>300000070</t>
+        </is>
       </c>
       <c r="E77" t="s">
         <v>308</v>
@@ -4957,8 +5070,10 @@
       <c r="J77" t="s">
         <v>21</v>
       </c>
-      <c r="L77" t="s">
-        <v>320</v>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>martinez.mirna@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="78" spans="1:12">
@@ -4971,8 +5086,10 @@
       <c r="C78" t="s">
         <v>306</v>
       </c>
-      <c r="D78" t="s">
-        <v>321</v>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>300000033</t>
+        </is>
       </c>
       <c r="E78" t="s">
         <v>155</v>
@@ -4983,8 +5100,10 @@
       <c r="I78" t="s">
         <v>42</v>
       </c>
-      <c r="L78" t="s">
-        <v>322</v>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>miranda.carlos@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="79" spans="1:12">
@@ -4997,8 +5116,10 @@
       <c r="C79" t="s">
         <v>306</v>
       </c>
-      <c r="D79" t="s">
-        <v>324</v>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>300000004</t>
+        </is>
       </c>
       <c r="E79" t="s">
         <v>36</v>
@@ -5009,8 +5130,10 @@
       <c r="I79" t="s">
         <v>42</v>
       </c>
-      <c r="L79" t="s">
-        <v>325</v>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>gutierrez.esther@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="80" spans="1:12">
@@ -5052,8 +5175,10 @@
       <c r="C81" t="s">
         <v>306</v>
       </c>
-      <c r="D81" t="s">
-        <v>329</v>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>300000078</t>
+        </is>
       </c>
       <c r="E81" t="s">
         <v>327</v>
@@ -5067,8 +5192,10 @@
       <c r="J81" t="s">
         <v>45</v>
       </c>
-      <c r="L81" t="s">
-        <v>330</v>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>zabala.nolberto@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="82" spans="1:12">
@@ -5081,8 +5208,10 @@
       <c r="C82" t="s">
         <v>306</v>
       </c>
-      <c r="D82" t="s">
-        <v>331</v>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>300000078</t>
+        </is>
       </c>
       <c r="E82" t="s">
         <v>327</v>
@@ -5096,8 +5225,10 @@
       <c r="J82" t="s">
         <v>332</v>
       </c>
-      <c r="L82" t="s">
-        <v>333</v>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>zabala.nolberto@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="83" spans="1:12">
@@ -5110,8 +5241,10 @@
       <c r="C83" t="s">
         <v>335</v>
       </c>
-      <c r="D83" t="s">
-        <v>336</v>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>300000054</t>
+        </is>
       </c>
       <c r="E83" t="s">
         <v>246</v>
@@ -5122,8 +5255,10 @@
       <c r="I83" t="s">
         <v>272</v>
       </c>
-      <c r="L83" t="s">
-        <v>337</v>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>terrazas.ricardo@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="84" spans="1:12">
@@ -5136,8 +5271,10 @@
       <c r="C84" t="s">
         <v>335</v>
       </c>
-      <c r="D84" t="s">
-        <v>338</v>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>300000002</t>
+        </is>
       </c>
       <c r="E84" t="s">
         <v>25</v>
@@ -5148,8 +5285,10 @@
       <c r="I84" t="s">
         <v>42</v>
       </c>
-      <c r="L84" t="s">
-        <v>339</v>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>cabello.ruben@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="85" spans="1:12">
@@ -5281,8 +5420,10 @@
       <c r="C89" t="s">
         <v>341</v>
       </c>
-      <c r="D89" t="s">
-        <v>356</v>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>300000086</t>
+        </is>
       </c>
       <c r="E89" t="s">
         <v>354</v>
@@ -5296,8 +5437,10 @@
       <c r="J89" t="s">
         <v>357</v>
       </c>
-      <c r="L89" t="s">
-        <v>358</v>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>cayoja.milton@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="90" spans="1:12">
@@ -5437,8 +5580,10 @@
       <c r="C95" t="s">
         <v>341</v>
       </c>
-      <c r="D95" t="s">
-        <v>377</v>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>300000040</t>
+        </is>
       </c>
       <c r="E95" t="s">
         <v>184</v>
@@ -5452,8 +5597,10 @@
       <c r="I95" t="s">
         <v>75</v>
       </c>
-      <c r="L95" t="s">
-        <v>378</v>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>lazo.roberto@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="96" spans="1:12">
@@ -5530,8 +5677,10 @@
       <c r="C98" t="s">
         <v>386</v>
       </c>
-      <c r="D98" t="s">
-        <v>387</v>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>300000085</t>
+        </is>
       </c>
       <c r="E98" t="s">
         <v>351</v>
@@ -5545,8 +5694,10 @@
       <c r="I98" t="s">
         <v>75</v>
       </c>
-      <c r="L98" t="s">
-        <v>388</v>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>calderon.franklin@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="99" spans="1:12">
@@ -5559,8 +5710,10 @@
       <c r="C99" t="s">
         <v>386</v>
       </c>
-      <c r="D99" t="s">
-        <v>389</v>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>300000085</t>
+        </is>
       </c>
       <c r="E99" t="s">
         <v>351</v>
@@ -5574,8 +5727,10 @@
       <c r="J99" t="s">
         <v>37</v>
       </c>
-      <c r="L99" t="s">
-        <v>390</v>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>calderon.franklin@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="100" spans="1:12">
@@ -5617,8 +5772,10 @@
       <c r="C101" t="s">
         <v>386</v>
       </c>
-      <c r="D101" t="s">
-        <v>394</v>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>300000098</t>
+        </is>
       </c>
       <c r="E101" t="s">
         <v>392</v>
@@ -5632,8 +5789,10 @@
       <c r="J101" t="s">
         <v>332</v>
       </c>
-      <c r="L101" t="s">
-        <v>395</v>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>zeballos.luis@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="102" spans="1:12">
@@ -5646,8 +5805,10 @@
       <c r="C102" t="s">
         <v>386</v>
       </c>
-      <c r="D102" t="s">
-        <v>397</v>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>300000098</t>
+        </is>
       </c>
       <c r="E102" t="s">
         <v>392</v>
@@ -5661,8 +5822,10 @@
       <c r="J102" t="s">
         <v>17</v>
       </c>
-      <c r="L102" t="s">
-        <v>398</v>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>zeballos.luis@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="103" spans="1:12">
@@ -5762,8 +5925,10 @@
       <c r="C106" t="s">
         <v>404</v>
       </c>
-      <c r="D106" t="s">
-        <v>411</v>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>300000052</t>
+        </is>
       </c>
       <c r="E106" t="s">
         <v>236</v>
@@ -5777,8 +5942,10 @@
       <c r="J106" t="s">
         <v>220</v>
       </c>
-      <c r="L106" t="s">
-        <v>412</v>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>salvatierra.rolando@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="107" spans="1:12">
@@ -5872,8 +6039,10 @@
       <c r="C110" t="s">
         <v>425</v>
       </c>
-      <c r="D110" t="s">
-        <v>429</v>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>300000107</t>
+        </is>
       </c>
       <c r="E110" t="s">
         <v>427</v>
@@ -5884,8 +6053,10 @@
       <c r="I110" t="s">
         <v>67</v>
       </c>
-      <c r="L110" t="s">
-        <v>430</v>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>martinez.antonio@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="111" spans="1:12">
@@ -5898,8 +6069,10 @@
       <c r="C111" t="s">
         <v>432</v>
       </c>
-      <c r="D111" t="s">
-        <v>433</v>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>300000107</t>
+        </is>
       </c>
       <c r="E111" t="s">
         <v>427</v>
@@ -5910,8 +6083,10 @@
       <c r="I111" t="s">
         <v>75</v>
       </c>
-      <c r="L111" t="s">
-        <v>434</v>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>martinez.antonio@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="112" spans="1:12">
@@ -5953,8 +6128,10 @@
       <c r="C113" t="s">
         <v>436</v>
       </c>
-      <c r="D113" t="s">
-        <v>440</v>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>300000110</t>
+        </is>
       </c>
       <c r="E113" t="s">
         <v>438</v>
@@ -5968,8 +6145,10 @@
       <c r="J113" t="s">
         <v>21</v>
       </c>
-      <c r="L113" t="s">
-        <v>441</v>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>claure.elizabeth@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="114" spans="1:12">
@@ -5982,8 +6161,10 @@
       <c r="C114" t="s">
         <v>436</v>
       </c>
-      <c r="D114" t="s">
-        <v>442</v>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>300000110</t>
+        </is>
       </c>
       <c r="E114" t="s">
         <v>438</v>
@@ -5994,8 +6175,10 @@
       <c r="I114" t="s">
         <v>160</v>
       </c>
-      <c r="L114" t="s">
-        <v>443</v>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>claure.elizabeth@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="115" spans="1:12">
@@ -6008,8 +6191,10 @@
       <c r="C115" t="s">
         <v>436</v>
       </c>
-      <c r="D115" t="s">
-        <v>444</v>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>300000110</t>
+        </is>
       </c>
       <c r="E115" t="s">
         <v>438</v>
@@ -6023,8 +6208,10 @@
       <c r="J115" t="s">
         <v>32</v>
       </c>
-      <c r="L115" t="s">
-        <v>445</v>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>claure.elizabeth@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="116" spans="1:12">
@@ -6066,8 +6253,10 @@
       <c r="C117" t="s">
         <v>450</v>
       </c>
-      <c r="D117" t="s">
-        <v>451</v>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>300000110</t>
+        </is>
       </c>
       <c r="E117" t="s">
         <v>438</v>
@@ -6081,8 +6270,10 @@
       <c r="J117" t="s">
         <v>45</v>
       </c>
-      <c r="L117" t="s">
-        <v>452</v>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>claure.elizabeth@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="118" spans="1:12">
@@ -6179,8 +6370,10 @@
       <c r="C121" t="s">
         <v>463</v>
       </c>
-      <c r="D121" t="s">
-        <v>464</v>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>300000069</t>
+        </is>
       </c>
       <c r="E121" t="s">
         <v>303</v>
@@ -6191,8 +6384,10 @@
       <c r="I121" t="s">
         <v>75</v>
       </c>
-      <c r="L121" t="s">
-        <v>465</v>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>vargas.edwin@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="122" spans="1:12">
@@ -6312,8 +6507,10 @@
       <c r="C126" t="s">
         <v>477</v>
       </c>
-      <c r="D126" t="s">
-        <v>484</v>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>300000018</t>
+        </is>
       </c>
       <c r="E126" t="s">
         <v>90</v>
@@ -6324,8 +6521,10 @@
       <c r="I126" t="s">
         <v>147</v>
       </c>
-      <c r="L126" t="s">
-        <v>485</v>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>veizaga.obed@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="127" spans="1:12">
@@ -6422,8 +6621,10 @@
       <c r="C130" t="s">
         <v>477</v>
       </c>
-      <c r="D130" t="s">
-        <v>496</v>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>300000063</t>
+        </is>
       </c>
       <c r="E130" t="s">
         <v>283</v>
@@ -6437,8 +6638,10 @@
       <c r="J130" t="s">
         <v>21</v>
       </c>
-      <c r="L130" t="s">
-        <v>497</v>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>lopez.milton@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="131" spans="1:12">
@@ -6451,8 +6654,10 @@
       <c r="C131" t="s">
         <v>477</v>
       </c>
-      <c r="D131" t="s">
-        <v>498</v>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>300000123</t>
+        </is>
       </c>
       <c r="E131" t="s">
         <v>482</v>
@@ -6466,8 +6671,10 @@
       <c r="J131" t="s">
         <v>37</v>
       </c>
-      <c r="L131" t="s">
-        <v>499</v>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>garzon.angelica@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="132" spans="1:12">
@@ -6480,8 +6687,10 @@
       <c r="C132" t="s">
         <v>477</v>
       </c>
-      <c r="D132" t="s">
-        <v>500</v>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>300000127</t>
+        </is>
       </c>
       <c r="E132" t="s">
         <v>494</v>
@@ -6495,8 +6704,10 @@
       <c r="J132" t="s">
         <v>332</v>
       </c>
-      <c r="L132" t="s">
-        <v>501</v>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>contreras.carlos@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="133" spans="1:12">
@@ -6509,8 +6720,10 @@
       <c r="C133" t="s">
         <v>477</v>
       </c>
-      <c r="D133" t="s">
-        <v>502</v>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>300000122</t>
+        </is>
       </c>
       <c r="E133" t="s">
         <v>479</v>
@@ -6524,8 +6737,10 @@
       <c r="J133" t="s">
         <v>17</v>
       </c>
-      <c r="L133" t="s">
-        <v>503</v>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>mollo.alberto@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="134" spans="1:12">
@@ -6538,8 +6753,10 @@
       <c r="C134" t="s">
         <v>477</v>
       </c>
-      <c r="D134" t="s">
-        <v>504</v>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>300000063</t>
+        </is>
       </c>
       <c r="E134" t="s">
         <v>283</v>
@@ -6550,8 +6767,10 @@
       <c r="I134" t="s">
         <v>147</v>
       </c>
-      <c r="L134" t="s">
-        <v>505</v>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>lopez.milton@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="135" spans="1:12">
@@ -6593,8 +6812,10 @@
       <c r="C136" t="s">
         <v>510</v>
       </c>
-      <c r="D136" t="s">
-        <v>511</v>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>300000126</t>
+        </is>
       </c>
       <c r="E136" t="s">
         <v>491</v>
@@ -6608,8 +6829,10 @@
       <c r="J136" t="s">
         <v>37</v>
       </c>
-      <c r="L136" t="s">
-        <v>512</v>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>zuna.ricardo@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="137" spans="1:12">
@@ -6622,8 +6845,10 @@
       <c r="C137" t="s">
         <v>510</v>
       </c>
-      <c r="D137" t="s">
-        <v>513</v>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>300000126</t>
+        </is>
       </c>
       <c r="E137" t="s">
         <v>491</v>
@@ -6637,8 +6862,10 @@
       <c r="J137" t="s">
         <v>220</v>
       </c>
-      <c r="L137" t="s">
-        <v>514</v>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>zuna.ricardo@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="138" spans="1:12">
@@ -6677,8 +6904,10 @@
       <c r="C139" t="s">
         <v>521</v>
       </c>
-      <c r="D139" t="s">
-        <v>522</v>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>300000084</t>
+        </is>
       </c>
       <c r="E139" t="s">
         <v>347</v>
@@ -6692,8 +6921,10 @@
       <c r="J139" t="s">
         <v>121</v>
       </c>
-      <c r="L139" t="s">
-        <v>523</v>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>sanchez.gabriel@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="140" spans="1:12">
@@ -6758,8 +6989,10 @@
       <c r="C142" t="s">
         <v>530</v>
       </c>
-      <c r="D142" t="s">
-        <v>534</v>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>300000084</t>
+        </is>
       </c>
       <c r="E142" t="s">
         <v>347</v>
@@ -6773,8 +7006,10 @@
       <c r="J142" t="s">
         <v>526</v>
       </c>
-      <c r="L142" t="s">
-        <v>535</v>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>sanchez.gabriel@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="143" spans="1:12">
@@ -6813,8 +7048,10 @@
       <c r="C144" t="s">
         <v>542</v>
       </c>
-      <c r="D144" t="s">
-        <v>543</v>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>300000083</t>
+        </is>
       </c>
       <c r="E144" t="s">
         <v>343</v>
@@ -6825,8 +7062,10 @@
       <c r="K144" t="s">
         <v>544</v>
       </c>
-      <c r="L144" t="s">
-        <v>545</v>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>lamas.rodrigo@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="145" spans="1:12">
@@ -6839,8 +7078,10 @@
       <c r="C145" t="s">
         <v>547</v>
       </c>
-      <c r="D145" t="s">
-        <v>548</v>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>300000033</t>
+        </is>
       </c>
       <c r="E145" t="s">
         <v>155</v>
@@ -6854,8 +7095,10 @@
       <c r="J145" t="s">
         <v>21</v>
       </c>
-      <c r="L145" t="s">
-        <v>549</v>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>miranda.carlos@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="146" spans="1:12">
@@ -6868,8 +7111,10 @@
       <c r="C146" t="s">
         <v>551</v>
       </c>
-      <c r="D146" t="s">
-        <v>552</v>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>300000121</t>
+        </is>
       </c>
       <c r="E146" t="s">
         <v>474</v>
@@ -6880,8 +7125,10 @@
       <c r="I146" t="s">
         <v>45</v>
       </c>
-      <c r="L146" t="s">
-        <v>553</v>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>rissiotti.zacarias@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="147" spans="1:12">
@@ -6894,8 +7141,10 @@
       <c r="C147" t="s">
         <v>555</v>
       </c>
-      <c r="D147" t="s">
-        <v>556</v>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>300000050</t>
+        </is>
       </c>
       <c r="E147" t="s">
         <v>225</v>
@@ -6906,8 +7155,10 @@
       <c r="I147" t="s">
         <v>344</v>
       </c>
-      <c r="L147" t="s">
-        <v>557</v>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>perez.eulalia@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="148" spans="1:12">
@@ -6943,8 +7194,10 @@
       <c r="C149" t="s">
         <v>555</v>
       </c>
-      <c r="D149" t="s">
-        <v>561</v>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>300000038</t>
+        </is>
       </c>
       <c r="E149" t="s">
         <v>176</v>
@@ -6955,8 +7208,10 @@
       <c r="I149" t="s">
         <v>17</v>
       </c>
-      <c r="L149" t="s">
-        <v>562</v>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>oropeza.adolfo@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="150" spans="1:12">
@@ -6995,8 +7250,10 @@
       <c r="C151" t="s">
         <v>567</v>
       </c>
-      <c r="D151" t="s">
-        <v>568</v>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>300000062</t>
+        </is>
       </c>
       <c r="E151" t="s">
         <v>278</v>
@@ -7007,8 +7264,10 @@
       <c r="I151" t="s">
         <v>42</v>
       </c>
-      <c r="L151" t="s">
-        <v>569</v>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>gianella.antonio@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="152" spans="1:12">
@@ -7021,8 +7280,10 @@
       <c r="C152" t="s">
         <v>567</v>
       </c>
-      <c r="D152" t="s">
-        <v>570</v>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>300000005</t>
+        </is>
       </c>
       <c r="E152" t="s">
         <v>41</v>
@@ -7033,8 +7294,10 @@
       <c r="J152" t="s">
         <v>147</v>
       </c>
-      <c r="L152" t="s">
-        <v>571</v>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>gianella.eduardo@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="153" spans="1:12">
@@ -7047,8 +7310,10 @@
       <c r="C153" t="s">
         <v>567</v>
       </c>
-      <c r="D153" t="s">
-        <v>572</v>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>300000062</t>
+        </is>
       </c>
       <c r="E153" t="s">
         <v>278</v>
@@ -7059,8 +7324,10 @@
       <c r="I153" t="s">
         <v>147</v>
       </c>
-      <c r="L153" t="s">
-        <v>573</v>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>gianella.antonio@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="154" spans="1:12">
@@ -7099,8 +7366,10 @@
       <c r="C155" t="s">
         <v>579</v>
       </c>
-      <c r="D155" t="s">
-        <v>580</v>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>300000054</t>
+        </is>
       </c>
       <c r="E155" t="s">
         <v>246</v>
@@ -7111,8 +7380,10 @@
       <c r="I155" t="s">
         <v>147</v>
       </c>
-      <c r="L155" t="s">
-        <v>581</v>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>terrazas.ricardo@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="156" spans="1:12">
@@ -7125,8 +7396,10 @@
       <c r="C156" t="s">
         <v>579</v>
       </c>
-      <c r="D156" t="s">
-        <v>582</v>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>300000002</t>
+        </is>
       </c>
       <c r="E156" t="s">
         <v>25</v>
@@ -7140,8 +7413,10 @@
       <c r="J156" t="s">
         <v>37</v>
       </c>
-      <c r="L156" t="s">
-        <v>583</v>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>cabello.ruben@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="157" spans="1:12">
@@ -7180,8 +7455,10 @@
       <c r="C158" t="s">
         <v>591</v>
       </c>
-      <c r="D158" t="s">
-        <v>592</v>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>300000004</t>
+        </is>
       </c>
       <c r="E158" t="s">
         <v>36</v>
@@ -7192,8 +7469,10 @@
       <c r="I158" t="s">
         <v>147</v>
       </c>
-      <c r="L158" t="s">
-        <v>593</v>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>gutierrez.esther@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="159" spans="1:12">
@@ -7206,8 +7485,10 @@
       <c r="C159" t="s">
         <v>591</v>
       </c>
-      <c r="D159" t="s">
-        <v>594</v>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>300000023</t>
+        </is>
       </c>
       <c r="E159" t="s">
         <v>111</v>
@@ -7218,8 +7499,10 @@
       <c r="J159" t="s">
         <v>42</v>
       </c>
-      <c r="L159" t="s">
-        <v>595</v>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>perez.ubaldo@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="160" spans="1:12">
@@ -7232,8 +7515,10 @@
       <c r="C160" t="s">
         <v>597</v>
       </c>
-      <c r="D160" t="s">
-        <v>598</v>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>300000089</t>
+        </is>
       </c>
       <c r="E160" t="s">
         <v>365</v>
@@ -7244,8 +7529,10 @@
       <c r="I160" t="s">
         <v>147</v>
       </c>
-      <c r="L160" t="s">
-        <v>599</v>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>cano.jorge@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="161" spans="1:12">
@@ -7313,8 +7600,10 @@
       <c r="C163" t="s">
         <v>597</v>
       </c>
-      <c r="D163" t="s">
-        <v>606</v>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>300000160</t>
+        </is>
       </c>
       <c r="E163" t="s">
         <v>604</v>
@@ -7325,8 +7614,10 @@
       <c r="I163" t="s">
         <v>607</v>
       </c>
-      <c r="L163" t="s">
-        <v>608</v>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>sanchez.alejandro@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="164" spans="1:12">
@@ -7365,8 +7656,10 @@
       <c r="C165" t="s">
         <v>613</v>
       </c>
-      <c r="D165" t="s">
-        <v>614</v>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>300000089</t>
+        </is>
       </c>
       <c r="E165" t="s">
         <v>365</v>
@@ -7377,8 +7670,10 @@
       <c r="H165" t="s">
         <v>147</v>
       </c>
-      <c r="L165" t="s">
-        <v>615</v>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>cano.jorge@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="166" spans="1:12">
@@ -7391,8 +7686,10 @@
       <c r="C166" t="s">
         <v>613</v>
       </c>
-      <c r="D166" t="s">
-        <v>616</v>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>300000160</t>
+        </is>
       </c>
       <c r="E166" t="s">
         <v>604</v>
@@ -7406,8 +7703,10 @@
       <c r="J166" t="s">
         <v>37</v>
       </c>
-      <c r="L166" t="s">
-        <v>617</v>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>sanchez.alejandro@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="167" spans="1:12">
@@ -7504,8 +7803,10 @@
       <c r="C170" t="s">
         <v>627</v>
       </c>
-      <c r="D170" t="s">
-        <v>631</v>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>300000167</t>
+        </is>
       </c>
       <c r="E170" t="s">
         <v>629</v>
@@ -7516,8 +7817,10 @@
       <c r="I170" t="s">
         <v>42</v>
       </c>
-      <c r="L170" t="s">
-        <v>632</v>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>vallet.corrado@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="171" spans="1:12">
@@ -7556,8 +7859,10 @@
       <c r="C172" t="s">
         <v>627</v>
       </c>
-      <c r="D172" t="s">
-        <v>637</v>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>300000167</t>
+        </is>
       </c>
       <c r="E172" t="s">
         <v>629</v>
@@ -7571,8 +7876,10 @@
       <c r="J172" t="s">
         <v>37</v>
       </c>
-      <c r="L172" t="s">
-        <v>638</v>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>vallet.corrado@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="173" spans="1:12">
@@ -7608,8 +7915,10 @@
       <c r="C174" t="s">
         <v>646</v>
       </c>
-      <c r="D174" t="s">
-        <v>647</v>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>300000122</t>
+        </is>
       </c>
       <c r="E174" t="s">
         <v>479</v>
@@ -7620,8 +7929,10 @@
       <c r="I174" t="s">
         <v>42</v>
       </c>
-      <c r="L174" t="s">
-        <v>648</v>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t>mollo.alberto@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="175" spans="1:12">
@@ -7634,8 +7945,10 @@
       <c r="C175" t="s">
         <v>646</v>
       </c>
-      <c r="D175" t="s">
-        <v>649</v>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>300000069</t>
+        </is>
       </c>
       <c r="E175" t="s">
         <v>303</v>
@@ -7649,8 +7962,10 @@
       <c r="J175" t="s">
         <v>96</v>
       </c>
-      <c r="L175" t="s">
-        <v>650</v>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>vargas.edwin@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="176" spans="1:12">
@@ -7692,8 +8007,10 @@
       <c r="C177" t="s">
         <v>646</v>
       </c>
-      <c r="D177" t="s">
-        <v>654</v>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>300000122</t>
+        </is>
       </c>
       <c r="E177" t="s">
         <v>479</v>
@@ -7707,8 +8024,10 @@
       <c r="J177" t="s">
         <v>21</v>
       </c>
-      <c r="L177" t="s">
-        <v>655</v>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>mollo.alberto@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="178" spans="1:12">
@@ -7721,8 +8040,10 @@
       <c r="C178" t="s">
         <v>646</v>
       </c>
-      <c r="D178" t="s">
-        <v>656</v>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>300000174</t>
+        </is>
       </c>
       <c r="E178" t="s">
         <v>652</v>
@@ -7736,8 +8057,10 @@
       <c r="J178" t="s">
         <v>21</v>
       </c>
-      <c r="L178" t="s">
-        <v>657</v>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>balcazar.evans@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="179" spans="1:12">
@@ -7750,8 +8073,10 @@
       <c r="C179" t="s">
         <v>646</v>
       </c>
-      <c r="D179" t="s">
-        <v>658</v>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>300000122</t>
+        </is>
       </c>
       <c r="E179" t="s">
         <v>479</v>
@@ -7765,8 +8090,10 @@
       <c r="J179" t="s">
         <v>121</v>
       </c>
-      <c r="L179" t="s">
-        <v>659</v>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>mollo.alberto@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="180" spans="1:12">
@@ -7805,8 +8132,10 @@
       <c r="C181" t="s">
         <v>646</v>
       </c>
-      <c r="D181" t="s">
-        <v>663</v>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>300000178</t>
+        </is>
       </c>
       <c r="E181" t="s">
         <v>661</v>
@@ -7820,8 +8149,10 @@
       <c r="J181" t="s">
         <v>96</v>
       </c>
-      <c r="L181" t="s">
-        <v>664</v>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>acosta.hugo@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="182" spans="1:12">
@@ -7834,8 +8165,10 @@
       <c r="C182" t="s">
         <v>666</v>
       </c>
-      <c r="D182" t="s">
-        <v>667</v>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>300000127</t>
+        </is>
       </c>
       <c r="E182" t="s">
         <v>494</v>
@@ -7846,8 +8179,10 @@
       <c r="I182" t="s">
         <v>160</v>
       </c>
-      <c r="L182" t="s">
-        <v>668</v>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>contreras.carlos@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="183" spans="1:12">
@@ -7860,8 +8195,10 @@
       <c r="C183" t="s">
         <v>666</v>
       </c>
-      <c r="D183" t="s">
-        <v>669</v>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>300000127</t>
+        </is>
       </c>
       <c r="E183" t="s">
         <v>494</v>
@@ -7872,8 +8209,10 @@
       <c r="I183" t="s">
         <v>147</v>
       </c>
-      <c r="L183" t="s">
-        <v>670</v>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>contreras.carlos@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="184" spans="1:12">
@@ -7886,8 +8225,10 @@
       <c r="C184" t="s">
         <v>666</v>
       </c>
-      <c r="D184" t="s">
-        <v>671</v>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>300000127</t>
+        </is>
       </c>
       <c r="E184" t="s">
         <v>494</v>
@@ -7898,8 +8239,10 @@
       <c r="I184" t="s">
         <v>42</v>
       </c>
-      <c r="L184" t="s">
-        <v>672</v>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>contreras.carlos@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="185" spans="1:12">
@@ -7912,8 +8255,10 @@
       <c r="C185" t="s">
         <v>666</v>
       </c>
-      <c r="D185" t="s">
-        <v>673</v>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>300000050</t>
+        </is>
       </c>
       <c r="E185" t="s">
         <v>225</v>
@@ -7927,8 +8272,10 @@
       <c r="J185" t="s">
         <v>80</v>
       </c>
-      <c r="L185" t="s">
-        <v>674</v>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t>perez.eulalia@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="186" spans="1:12">
@@ -7967,8 +8314,10 @@
       <c r="C187" t="s">
         <v>679</v>
       </c>
-      <c r="D187" t="s">
-        <v>680</v>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>300000046</t>
+        </is>
       </c>
       <c r="E187" t="s">
         <v>207</v>
@@ -7979,8 +8328,10 @@
       <c r="I187" t="s">
         <v>75</v>
       </c>
-      <c r="L187" t="s">
-        <v>681</v>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>barroso.gino@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="188" spans="1:12">
@@ -7993,8 +8344,10 @@
       <c r="C188" t="s">
         <v>683</v>
       </c>
-      <c r="D188" t="s">
-        <v>684</v>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>300000078</t>
+        </is>
       </c>
       <c r="E188" t="s">
         <v>327</v>
@@ -8005,8 +8358,10 @@
       <c r="I188" t="s">
         <v>526</v>
       </c>
-      <c r="L188" t="s">
-        <v>685</v>
+      <c r="L188" t="inlineStr">
+        <is>
+          <t>zabala.nolberto@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="189" spans="1:12">
@@ -8074,8 +8429,10 @@
       <c r="C191" t="s">
         <v>687</v>
       </c>
-      <c r="D191" t="s">
-        <v>694</v>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>300000009</t>
+        </is>
       </c>
       <c r="E191" t="s">
         <v>54</v>
@@ -8086,8 +8443,10 @@
       <c r="I191" t="s">
         <v>147</v>
       </c>
-      <c r="L191" t="s">
-        <v>695</v>
+      <c r="L191" t="inlineStr">
+        <is>
+          <t>monrroy.fernando@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="192" spans="1:12">
@@ -8100,8 +8459,10 @@
       <c r="C192" t="s">
         <v>697</v>
       </c>
-      <c r="D192" t="s">
-        <v>698</v>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>300000187</t>
+        </is>
       </c>
       <c r="E192" t="s">
         <v>689</v>
@@ -8112,8 +8473,10 @@
       <c r="I192" t="s">
         <v>75</v>
       </c>
-      <c r="L192" t="s">
-        <v>699</v>
+      <c r="L192" t="inlineStr">
+        <is>
+          <t>gonzales.antonio@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="193" spans="1:12">
@@ -8126,8 +8489,10 @@
       <c r="C193" t="s">
         <v>697</v>
       </c>
-      <c r="D193" t="s">
-        <v>700</v>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>300000187</t>
+        </is>
       </c>
       <c r="E193" t="s">
         <v>689</v>
@@ -8141,8 +8506,10 @@
       <c r="J193" t="s">
         <v>17</v>
       </c>
-      <c r="L193" t="s">
-        <v>701</v>
+      <c r="L193" t="inlineStr">
+        <is>
+          <t>gonzales.antonio@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="194" spans="1:12">
@@ -8210,8 +8577,10 @@
       <c r="C196" t="s">
         <v>711</v>
       </c>
-      <c r="D196" t="s">
-        <v>712</v>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>300000174</t>
+        </is>
       </c>
       <c r="E196" t="s">
         <v>652</v>
@@ -8222,8 +8591,10 @@
       <c r="I196" t="s">
         <v>147</v>
       </c>
-      <c r="L196" t="s">
-        <v>713</v>
+      <c r="L196" t="inlineStr">
+        <is>
+          <t>balcazar.evans@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="197" spans="1:12">
@@ -8317,8 +8688,10 @@
       <c r="C200" t="s">
         <v>732</v>
       </c>
-      <c r="D200" t="s">
-        <v>733</v>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>300000060</t>
+        </is>
       </c>
       <c r="E200" t="s">
         <v>267</v>
@@ -8329,8 +8702,10 @@
       <c r="I200" t="s">
         <v>734</v>
       </c>
-      <c r="L200" t="s">
-        <v>735</v>
+      <c r="L200" t="inlineStr">
+        <is>
+          <t>rosales.marcelo@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="201" spans="1:12">
@@ -8343,8 +8718,10 @@
       <c r="C201" t="s">
         <v>737</v>
       </c>
-      <c r="D201" t="s">
-        <v>738</v>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>300000085</t>
+        </is>
       </c>
       <c r="E201" t="s">
         <v>351</v>
@@ -8358,8 +8735,10 @@
       <c r="J201" t="s">
         <v>17</v>
       </c>
-      <c r="L201" t="s">
-        <v>739</v>
+      <c r="L201" t="inlineStr">
+        <is>
+          <t>calderon.franklin@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="202" spans="1:12">
@@ -8372,8 +8751,10 @@
       <c r="C202" t="s">
         <v>737</v>
       </c>
-      <c r="D202" t="s">
-        <v>740</v>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>300000023</t>
+        </is>
       </c>
       <c r="E202" t="s">
         <v>111</v>
@@ -8384,8 +8765,10 @@
       <c r="I202" t="s">
         <v>741</v>
       </c>
-      <c r="L202" t="s">
-        <v>742</v>
+      <c r="L202" t="inlineStr">
+        <is>
+          <t>perez.ubaldo@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="203" spans="1:12">
@@ -8398,8 +8781,10 @@
       <c r="C203" t="s">
         <v>744</v>
       </c>
-      <c r="D203" t="s">
-        <v>745</v>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>300000123</t>
+        </is>
       </c>
       <c r="E203" t="s">
         <v>482</v>
@@ -8413,8 +8798,10 @@
       <c r="J203" t="s">
         <v>21</v>
       </c>
-      <c r="L203" t="s">
-        <v>746</v>
+      <c r="L203" t="inlineStr">
+        <is>
+          <t>garzon.angelica@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="204" spans="1:12">
@@ -8427,8 +8814,10 @@
       <c r="C204" t="s">
         <v>744</v>
       </c>
-      <c r="D204" t="s">
-        <v>747</v>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>300000123</t>
+        </is>
       </c>
       <c r="E204" t="s">
         <v>482</v>
@@ -8439,8 +8828,10 @@
       <c r="I204" t="s">
         <v>147</v>
       </c>
-      <c r="L204" t="s">
-        <v>748</v>
+      <c r="L204" t="inlineStr">
+        <is>
+          <t>garzon.angelica@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="205" spans="1:12">
@@ -8453,8 +8844,10 @@
       <c r="C205" t="s">
         <v>750</v>
       </c>
-      <c r="D205" t="s">
-        <v>751</v>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>300000123</t>
+        </is>
       </c>
       <c r="E205" t="s">
         <v>482</v>
@@ -8465,8 +8858,10 @@
       <c r="I205" t="s">
         <v>42</v>
       </c>
-      <c r="L205" t="s">
-        <v>752</v>
+      <c r="L205" t="inlineStr">
+        <is>
+          <t>garzon.angelica@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="206" spans="1:12">
@@ -8479,8 +8874,10 @@
       <c r="C206" t="s">
         <v>750</v>
       </c>
-      <c r="D206" t="s">
-        <v>753</v>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>300000107</t>
+        </is>
       </c>
       <c r="E206" t="s">
         <v>427</v>
@@ -8494,8 +8891,10 @@
       <c r="J206" t="s">
         <v>96</v>
       </c>
-      <c r="L206" t="s">
-        <v>754</v>
+      <c r="L206" t="inlineStr">
+        <is>
+          <t>martinez.antonio@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="207" spans="1:12">
@@ -8508,8 +8907,10 @@
       <c r="C207" t="s">
         <v>756</v>
       </c>
-      <c r="D207" t="s">
-        <v>757</v>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>300000046</t>
+        </is>
       </c>
       <c r="E207" t="s">
         <v>207</v>
@@ -8523,8 +8924,10 @@
       <c r="J207" t="s">
         <v>37</v>
       </c>
-      <c r="L207" t="s">
-        <v>758</v>
+      <c r="L207" t="inlineStr">
+        <is>
+          <t>barroso.gino@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="208" spans="1:12">
@@ -8563,8 +8966,10 @@
       <c r="C209" t="s">
         <v>766</v>
       </c>
-      <c r="D209" t="s">
-        <v>767</v>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>300000013</t>
+        </is>
       </c>
       <c r="E209" t="s">
         <v>72</v>
@@ -8575,8 +8980,10 @@
       <c r="J209" t="s">
         <v>272</v>
       </c>
-      <c r="L209" t="s">
-        <v>768</v>
+      <c r="L209" t="inlineStr">
+        <is>
+          <t>hinojosa.said@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="210" spans="1:12">
@@ -8589,8 +8996,10 @@
       <c r="C210" t="s">
         <v>770</v>
       </c>
-      <c r="D210" t="s">
-        <v>771</v>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>300000046</t>
+        </is>
       </c>
       <c r="E210" t="s">
         <v>207</v>
@@ -8604,8 +9013,10 @@
       <c r="J210" t="s">
         <v>21</v>
       </c>
-      <c r="L210" t="s">
-        <v>772</v>
+      <c r="L210" t="inlineStr">
+        <is>
+          <t>barroso.gino@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="211" spans="1:12">
@@ -8618,8 +9029,10 @@
       <c r="C211" t="s">
         <v>770</v>
       </c>
-      <c r="D211" t="s">
-        <v>773</v>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>300000046</t>
+        </is>
       </c>
       <c r="E211" t="s">
         <v>207</v>
@@ -8633,8 +9046,10 @@
       <c r="J211" t="s">
         <v>45</v>
       </c>
-      <c r="L211" t="s">
-        <v>774</v>
+      <c r="L211" t="inlineStr">
+        <is>
+          <t>barroso.gino@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="212" spans="1:12">
@@ -8647,14 +9062,18 @@
       <c r="C212" t="s">
         <v>770</v>
       </c>
-      <c r="D212" t="s">
-        <v>776</v>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>300000106</t>
+        </is>
       </c>
       <c r="E212" t="s">
         <v>421</v>
       </c>
-      <c r="L212" t="s">
-        <v>777</v>
+      <c r="L212" t="inlineStr">
+        <is>
+          <t>calle.edwin@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="213" spans="1:12">
@@ -8667,8 +9086,10 @@
       <c r="C213" t="s">
         <v>779</v>
       </c>
-      <c r="D213" t="s">
-        <v>780</v>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>300000088</t>
+        </is>
       </c>
       <c r="E213" t="s">
         <v>361</v>
@@ -8682,8 +9103,10 @@
       <c r="J213" t="s">
         <v>45</v>
       </c>
-      <c r="L213" t="s">
-        <v>781</v>
+      <c r="L213" t="inlineStr">
+        <is>
+          <t>sanchez.enrique@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="214" spans="1:12">
@@ -8696,8 +9119,10 @@
       <c r="C214" t="s">
         <v>779</v>
       </c>
-      <c r="D214" t="s">
-        <v>782</v>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>300000106</t>
+        </is>
       </c>
       <c r="E214" t="s">
         <v>421</v>
@@ -8708,8 +9133,10 @@
       <c r="I214" t="s">
         <v>67</v>
       </c>
-      <c r="L214" t="s">
-        <v>783</v>
+      <c r="L214" t="inlineStr">
+        <is>
+          <t>calle.edwin@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="215" spans="1:12">
@@ -8722,8 +9149,10 @@
       <c r="C215" t="s">
         <v>785</v>
       </c>
-      <c r="D215" t="s">
-        <v>786</v>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>300000094</t>
+        </is>
       </c>
       <c r="E215" t="s">
         <v>380</v>
@@ -8737,8 +9166,10 @@
       <c r="J215" t="s">
         <v>17</v>
       </c>
-      <c r="L215" t="s">
-        <v>787</v>
+      <c r="L215" t="inlineStr">
+        <is>
+          <t>aranibar.monica@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="216" spans="1:12">
@@ -8751,8 +9182,10 @@
       <c r="C216" t="s">
         <v>789</v>
       </c>
-      <c r="D216" t="s">
-        <v>790</v>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>300000187</t>
+        </is>
       </c>
       <c r="E216" t="s">
         <v>689</v>
@@ -8766,8 +9199,10 @@
       <c r="J216" t="s">
         <v>526</v>
       </c>
-      <c r="L216" t="s">
-        <v>791</v>
+      <c r="L216" t="inlineStr">
+        <is>
+          <t>gonzales.antonio@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="217" spans="1:12">
@@ -8780,8 +9215,10 @@
       <c r="C217" t="s">
         <v>793</v>
       </c>
-      <c r="D217" t="s">
-        <v>794</v>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>300000107</t>
+        </is>
       </c>
       <c r="E217" t="s">
         <v>427</v>
@@ -8792,8 +9229,10 @@
       <c r="I217" t="s">
         <v>260</v>
       </c>
-      <c r="L217" t="s">
-        <v>795</v>
+      <c r="L217" t="inlineStr">
+        <is>
+          <t>martinez.antonio@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="218" spans="1:12">
@@ -8835,8 +9274,10 @@
       <c r="C219" t="s">
         <v>793</v>
       </c>
-      <c r="D219" t="s">
-        <v>799</v>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>300000188</t>
+        </is>
       </c>
       <c r="E219" t="s">
         <v>692</v>
@@ -8850,8 +9291,10 @@
       <c r="J219" t="s">
         <v>121</v>
       </c>
-      <c r="L219" t="s">
-        <v>800</v>
+      <c r="L219" t="inlineStr">
+        <is>
+          <t>villagomez.junior@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="220" spans="1:12">
@@ -8893,8 +9336,10 @@
       <c r="C221" t="s">
         <v>807</v>
       </c>
-      <c r="D221" t="s">
-        <v>808</v>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>300000174</t>
+        </is>
       </c>
       <c r="E221" t="s">
         <v>652</v>
@@ -8905,8 +9350,10 @@
       <c r="I221" t="s">
         <v>42</v>
       </c>
-      <c r="L221" t="s">
-        <v>809</v>
+      <c r="L221" t="inlineStr">
+        <is>
+          <t>balcazar.evans@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="222" spans="1:12">
@@ -8919,8 +9366,10 @@
       <c r="C222" t="s">
         <v>807</v>
       </c>
-      <c r="D222" t="s">
-        <v>810</v>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>300000174</t>
+        </is>
       </c>
       <c r="E222" t="s">
         <v>652</v>
@@ -8934,8 +9383,10 @@
       <c r="J222" t="s">
         <v>45</v>
       </c>
-      <c r="L222" t="s">
-        <v>811</v>
+      <c r="L222" t="inlineStr">
+        <is>
+          <t>balcazar.evans@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="223" spans="1:12">
@@ -8948,14 +9399,18 @@
       <c r="C223" t="s">
         <v>813</v>
       </c>
-      <c r="D223" t="s">
-        <v>814</v>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>300000060</t>
+        </is>
       </c>
       <c r="E223" t="s">
         <v>267</v>
       </c>
-      <c r="L223" t="s">
-        <v>815</v>
+      <c r="L223" t="inlineStr">
+        <is>
+          <t>rosales.marcelo@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="224" spans="1:12">
@@ -8968,8 +9423,10 @@
       <c r="C224" t="s">
         <v>817</v>
       </c>
-      <c r="D224" t="s">
-        <v>818</v>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>300000052</t>
+        </is>
       </c>
       <c r="E224" t="s">
         <v>236</v>
@@ -8983,8 +9440,10 @@
       <c r="J224" t="s">
         <v>37</v>
       </c>
-      <c r="L224" t="s">
-        <v>819</v>
+      <c r="L224" t="inlineStr">
+        <is>
+          <t>salvatierra.rolando@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
     <row r="225" spans="1:12">
@@ -8997,8 +9456,10 @@
       <c r="C225" t="s">
         <v>821</v>
       </c>
-      <c r="D225" t="s">
-        <v>822</v>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>300000120</t>
+        </is>
       </c>
       <c r="E225" t="s">
         <v>469</v>
@@ -9009,8 +9470,10 @@
       <c r="I225" t="s">
         <v>75</v>
       </c>
-      <c r="L225" t="s">
-        <v>823</v>
+      <c r="L225" t="inlineStr">
+        <is>
+          <t>peinado.jesus@ficct.uagrm.edu.bo</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -9019,45 +9482,4 @@
     <ignoredError sqref="A1:L225" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" t="s">
-        <v>824</v>
-      </c>
-      <c r="B1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D1" t="s">
-        <v>825</v>
-      </c>
-      <c r="E1" t="s">
-        <v>826</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" t="s">
-        <v>827</v>
-      </c>
-      <c r="B2" t="s">
-        <v>828</v>
-      </c>
-      <c r="C2" t="s">
-        <v>829</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:E2" numberStoredAsText="1"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>